<commit_message>
fix: standardize Status Kepegawaian strictly to 4 types (PKWTT, PKWT, Probation, Magang)
</commit_message>
<xml_diff>
--- a/public/Template_Import_Karyawan_Gesit_People (1).xlsx
+++ b/public/Template_Import_Karyawan_Gesit_People (1).xlsx
@@ -588,7 +588,7 @@
         <v>1990-08-03</v>
       </c>
       <c r="Y2" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z2" t="str">
         <v>-</v>
@@ -701,7 +701,7 @@
         <v>1990-08-04</v>
       </c>
       <c r="Y3" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z3" t="str">
         <v>-</v>
@@ -814,7 +814,7 @@
         <v>1990-08-05</v>
       </c>
       <c r="Y4" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z4" t="str">
         <v>-</v>
@@ -927,7 +927,7 @@
         <v>1990-08-06</v>
       </c>
       <c r="Y5" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z5" t="str">
         <v>-</v>
@@ -1040,7 +1040,7 @@
         <v>1990-08-07</v>
       </c>
       <c r="Y6" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z6" t="str">
         <v>-</v>
@@ -1153,7 +1153,7 @@
         <v>2020-06-15</v>
       </c>
       <c r="Y7" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z7" t="str">
         <v>-</v>
@@ -1266,7 +1266,7 @@
         <v>2020-04-20</v>
       </c>
       <c r="Y8" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z8" t="str">
         <v>-</v>
@@ -1379,7 +1379,7 @@
         <v>2019-11-01</v>
       </c>
       <c r="Y9" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z9" t="str">
         <v>-</v>
@@ -1492,7 +1492,7 @@
         <v>1996-11-20</v>
       </c>
       <c r="Y10" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z10" t="str">
         <v>-</v>
@@ -1605,7 +1605,7 @@
         <v>1999-07-19</v>
       </c>
       <c r="Y11" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z11" t="str">
         <v>-</v>
@@ -1718,7 +1718,7 @@
         <v>1996-05-01</v>
       </c>
       <c r="Y12" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z12" t="str">
         <v>-</v>
@@ -1831,7 +1831,7 @@
         <v>1999-09-01</v>
       </c>
       <c r="Y13" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z13" t="str">
         <v>-</v>
@@ -1944,7 +1944,7 @@
         <v>1999-08-04</v>
       </c>
       <c r="Y14" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z14" t="str">
         <v>-</v>
@@ -2057,7 +2057,7 @@
         <v>2013-07-29</v>
       </c>
       <c r="Y15" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z15" t="str">
         <v>-</v>
@@ -2170,7 +2170,7 @@
         <v>1991-10-01</v>
       </c>
       <c r="Y16" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z16" t="str">
         <v>-</v>
@@ -2283,7 +2283,7 @@
         <v>2021-07-01</v>
       </c>
       <c r="Y17" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z17" t="str">
         <v>-</v>
@@ -2396,7 +2396,7 @@
         <v>2015-01-29</v>
       </c>
       <c r="Y18" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z18" t="str">
         <v>-</v>
@@ -2509,7 +2509,7 @@
         <v>2014-11-24</v>
       </c>
       <c r="Y19" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z19" t="str">
         <v>-</v>
@@ -2622,7 +2622,7 @@
         <v>2014-04-01</v>
       </c>
       <c r="Y20" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z20" t="str">
         <v>-</v>
@@ -2735,7 +2735,7 @@
         <v>2021-03-08</v>
       </c>
       <c r="Y21" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z21" t="str">
         <v>-</v>
@@ -2848,7 +2848,7 @@
         <v>2016-08-28</v>
       </c>
       <c r="Y22" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z22" t="str">
         <v>-</v>
@@ -2961,7 +2961,7 @@
         <v>2018-07-30</v>
       </c>
       <c r="Y23" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z23" t="str">
         <v>-</v>
@@ -3074,7 +3074,7 @@
         <v>2006-01-16</v>
       </c>
       <c r="Y24" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z24" t="str">
         <v>-</v>
@@ -3191,7 +3191,7 @@
         <v>1997-09-12</v>
       </c>
       <c r="Y25" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z25" t="str">
         <v>-</v>
@@ -3304,7 +3304,7 @@
         <v>2016-04-15</v>
       </c>
       <c r="Y26" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z26" t="str">
         <v>-</v>
@@ -3417,7 +3417,7 @@
         <v>2020-01-03</v>
       </c>
       <c r="Y27" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z27" t="str">
         <v>-</v>
@@ -3530,7 +3530,7 @@
         <v>2019-06-24</v>
       </c>
       <c r="Y28" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z28" t="str">
         <v>-</v>
@@ -3643,7 +3643,7 @@
         <v>2008-05-01</v>
       </c>
       <c r="Y29" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z29" t="str">
         <v>-</v>
@@ -3756,7 +3756,7 @@
         <v>2017-07-13</v>
       </c>
       <c r="Y30" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z30" t="str">
         <v>-</v>
@@ -3869,7 +3869,7 @@
         <v>2011-05-16</v>
       </c>
       <c r="Y31" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z31" t="str">
         <v>-</v>
@@ -3982,7 +3982,7 @@
         <v>2019-01-02</v>
       </c>
       <c r="Y32" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z32" t="str">
         <v>-</v>
@@ -4095,7 +4095,7 @@
         <v>2013-12-16</v>
       </c>
       <c r="Y33" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z33" t="str">
         <v>-</v>
@@ -4208,7 +4208,7 @@
         <v>2012-02-06</v>
       </c>
       <c r="Y34" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z34" t="str">
         <v>-</v>
@@ -4321,7 +4321,7 @@
         <v>1993-10-29</v>
       </c>
       <c r="Y35" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z35" t="str">
         <v>-</v>
@@ -4434,7 +4434,7 @@
         <v>2006-02-27</v>
       </c>
       <c r="Y36" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z36" t="str">
         <v>-</v>
@@ -4547,7 +4547,7 @@
         <v>2006-10-31</v>
       </c>
       <c r="Y37" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z37" t="str">
         <v>-</v>
@@ -4660,7 +4660,7 @@
         <v>2009-10-21</v>
       </c>
       <c r="Y38" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z38" t="str">
         <v>-</v>
@@ -4773,7 +4773,7 @@
         <v>2022-05-09</v>
       </c>
       <c r="Y39" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z39" t="str">
         <v>-</v>
@@ -4886,7 +4886,7 @@
         <v>2022-05-09</v>
       </c>
       <c r="Y40" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z40" t="str">
         <v>-</v>
@@ -4999,7 +4999,7 @@
         <v>2022-09-19</v>
       </c>
       <c r="Y41" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z41" t="str">
         <v>-</v>
@@ -5112,7 +5112,7 @@
         <v>2023-02-06</v>
       </c>
       <c r="Y42" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z42" t="str">
         <v>-</v>
@@ -5225,7 +5225,7 @@
         <v>2007-02-12</v>
       </c>
       <c r="Y43" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z43" t="str">
         <v>-</v>
@@ -5338,7 +5338,7 @@
         <v>2009-11-13</v>
       </c>
       <c r="Y44" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z44" t="str">
         <v>-</v>
@@ -5451,7 +5451,7 @@
         <v>2023-08-01</v>
       </c>
       <c r="Y45" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z45" t="str">
         <v>-</v>
@@ -5564,7 +5564,7 @@
         <v>2023-08-11</v>
       </c>
       <c r="Y46" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z46" t="str">
         <v>-</v>
@@ -5677,7 +5677,7 @@
         <v>2023-10-20</v>
       </c>
       <c r="Y47" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z47" t="str">
         <v>-</v>
@@ -5790,7 +5790,7 @@
         <v>2024-01-09</v>
       </c>
       <c r="Y48" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z48" t="str">
         <v>-</v>
@@ -5903,7 +5903,7 @@
         <v>2024-02-19</v>
       </c>
       <c r="Y49" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z49" t="str">
         <v>-</v>
@@ -6016,7 +6016,7 @@
         <v>2025-03-12</v>
       </c>
       <c r="Y50" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z50" t="str">
         <v>-</v>
@@ -6129,7 +6129,7 @@
         <v>2024-06-03</v>
       </c>
       <c r="Y51" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z51" t="str">
         <v>-</v>
@@ -6242,7 +6242,7 @@
         <v>2024-09-01</v>
       </c>
       <c r="Y52" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z52" t="str">
         <v>-</v>
@@ -6355,7 +6355,7 @@
         <v>2024-09-23</v>
       </c>
       <c r="Y53" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z53" t="str">
         <v>-</v>
@@ -6468,7 +6468,7 @@
         <v>2024-11-14</v>
       </c>
       <c r="Y54" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z54" t="str">
         <v>-</v>
@@ -6581,7 +6581,7 @@
         <v>2025-02-17</v>
       </c>
       <c r="Y55" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z55" t="str">
         <v>-</v>
@@ -6694,7 +6694,7 @@
         <v>2025-04-07</v>
       </c>
       <c r="Y56" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z56" t="str">
         <v>-</v>
@@ -6807,7 +6807,7 @@
         <v>2025-04-14</v>
       </c>
       <c r="Y57" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z57" t="str">
         <v>-</v>
@@ -6920,7 +6920,7 @@
         <v>2025-06-02</v>
       </c>
       <c r="Y58" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z58" t="str">
         <v>-</v>
@@ -7033,7 +7033,7 @@
         <v>2025-06-02</v>
       </c>
       <c r="Y59" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z59" t="str">
         <v>-</v>
@@ -7146,7 +7146,7 @@
         <v>2025-08-04</v>
       </c>
       <c r="Y60" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z60" t="str">
         <v>-</v>
@@ -7259,7 +7259,7 @@
         <v>2025-10-13</v>
       </c>
       <c r="Y61" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z61" t="str">
         <v>-</v>
@@ -7372,7 +7372,7 @@
         <v>2025-12-15</v>
       </c>
       <c r="Y62" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z62" t="str">
         <v>-</v>
@@ -7485,7 +7485,7 @@
         <v>2026-02-16</v>
       </c>
       <c r="Y63" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z63" t="str">
         <v>-</v>
@@ -7598,7 +7598,7 @@
         <v>2026-04-17</v>
       </c>
       <c r="Y64" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z64" t="str">
         <v>-</v>
@@ -7711,7 +7711,7 @@
         <v>2026-05-15</v>
       </c>
       <c r="Y65" t="str">
-        <v>Karyawan Tetap</v>
+        <v>PKWTT</v>
       </c>
       <c r="Z65" t="str">
         <v>-</v>
@@ -7824,7 +7824,7 @@
         <v>2026-05-18</v>
       </c>
       <c r="Y66" t="str">
-        <v>PKWT 1</v>
+        <v>PKWT</v>
       </c>
       <c r="Z66" t="str">
         <v>-</v>
@@ -7937,7 +7937,7 @@
         <v>2026-07-06</v>
       </c>
       <c r="Y67" t="str">
-        <v>PKWT 1</v>
+        <v>PKWT</v>
       </c>
       <c r="Z67" t="str">
         <v>-</v>
@@ -8050,7 +8050,7 @@
         <v>2026-07-08</v>
       </c>
       <c r="Y68" t="str">
-        <v>PKWT 1</v>
+        <v>PKWT</v>
       </c>
       <c r="Z68" t="str">
         <v>-</v>
@@ -8163,7 +8163,7 @@
         <v>2026-07-27</v>
       </c>
       <c r="Y69" t="str">
-        <v>PROBATION</v>
+        <v>Probation</v>
       </c>
       <c r="Z69" t="str">
         <v>-</v>
@@ -8276,7 +8276,7 @@
         <v>2026-08-10</v>
       </c>
       <c r="Y70" t="str">
-        <v>PROBATION</v>
+        <v>Probation</v>
       </c>
       <c r="Z70" t="str">
         <v>-</v>
@@ -8389,7 +8389,7 @@
         <v>2026-08-18</v>
       </c>
       <c r="Y71" t="str">
-        <v>PROBATION</v>
+        <v>Probation</v>
       </c>
       <c r="Z71" t="str">
         <v>-</v>
@@ -8502,7 +8502,7 @@
         <v>2026-08-20</v>
       </c>
       <c r="Y72" t="str">
-        <v>PROBATION</v>
+        <v>Probation</v>
       </c>
       <c r="Z72" t="str">
         <v>-</v>
@@ -8615,7 +8615,7 @@
         <v>2026-10-05</v>
       </c>
       <c r="Y73" t="str">
-        <v>PROBATION</v>
+        <v>Probation</v>
       </c>
       <c r="Z73" t="str">
         <v>-</v>
@@ -8728,7 +8728,7 @@
         <v>2026-09-21</v>
       </c>
       <c r="Y74" t="str">
-        <v>PKWT 1</v>
+        <v>PKWT</v>
       </c>
       <c r="Z74" t="str">
         <v>-</v>

</xml_diff>

<commit_message>
fix: standardize gender (Laki-laki/Perempuan), religion options, and format dates to DD/MM/YYYY
</commit_message>
<xml_diff>
--- a/public/Template_Import_Karyawan_Gesit_People (1).xlsx
+++ b/public/Template_Import_Karyawan_Gesit_People (1).xlsx
@@ -427,7 +427,7 @@
         <v>Tempat Lahir</v>
       </c>
       <c r="I1" t="str">
-        <v>Tanggal Lahir (YYYY-MM-DD)</v>
+        <v>Tanggal Lahir (DD/MM/YYYY)</v>
       </c>
       <c r="J1" t="str">
         <v>Jenis Kelamin (Laki-laki/Perempuan)</v>
@@ -472,19 +472,19 @@
         <v>Status Akun (Active/Disabled)</v>
       </c>
       <c r="X1" t="str">
-        <v>Tanggal Mulai Kerja (YYYY-MM-DD)</v>
+        <v>Tanggal Mulai Kerja (DD/MM/YYYY)</v>
       </c>
       <c r="Y1" t="str">
-        <v>Status Kontrak (Probation/PKWT 1/PKWT 2/Karyawan Tetap)</v>
+        <v>Status Kepegawaian (PKWTT/PKWT/Probation/Magang)</v>
       </c>
       <c r="Z1" t="str">
         <v>Nomor PKWT / SK Karyawan</v>
       </c>
       <c r="AA1" t="str">
-        <v>Tanggal Mulai Kontrak (YYYY-MM-DD)</v>
+        <v>Tanggal Mulai Kontrak (DD/MM/YYYY)</v>
       </c>
       <c r="AB1" t="str">
-        <v>Tanggal Selesai Kontrak (YYYY-MM-DD)</v>
+        <v>Tanggal Selesai Kontrak (DD/MM/YYYY)</v>
       </c>
       <c r="AC1" t="str">
         <v>Status Payroll (Active/Hold)</v>
@@ -540,13 +540,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I2" t="str">
-        <v>1956-09-26</v>
+        <v>26/09/1956</v>
       </c>
       <c r="J2" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K2" t="str">
-        <v>Catholic</v>
+        <v>Katolik</v>
       </c>
       <c r="L2" t="str">
         <v>Married</v>
@@ -585,7 +585,7 @@
         <v>Active</v>
       </c>
       <c r="X2" t="str">
-        <v>1990-08-03</v>
+        <v>03/08/1990</v>
       </c>
       <c r="Y2" t="str">
         <v>PKWTT</v>
@@ -594,7 +594,7 @@
         <v>-</v>
       </c>
       <c r="AA2" t="str">
-        <v>1990-08-03</v>
+        <v>03/08/1990</v>
       </c>
       <c r="AB2" t="str">
         <v/>
@@ -653,13 +653,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I3" t="str">
-        <v>1958-07-12</v>
+        <v>12/07/1958</v>
       </c>
       <c r="J3" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K3" t="str">
-        <v>Catholic</v>
+        <v>Katolik</v>
       </c>
       <c r="L3" t="str">
         <v>Married</v>
@@ -698,7 +698,7 @@
         <v>Active</v>
       </c>
       <c r="X3" t="str">
-        <v>1990-08-04</v>
+        <v>04/08/1990</v>
       </c>
       <c r="Y3" t="str">
         <v>PKWTT</v>
@@ -707,7 +707,7 @@
         <v>-</v>
       </c>
       <c r="AA3" t="str">
-        <v>1990-08-04</v>
+        <v>04/08/1990</v>
       </c>
       <c r="AB3" t="str">
         <v/>
@@ -766,13 +766,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I4" t="str">
-        <v>1955-01-06</v>
+        <v>06/01/1955</v>
       </c>
       <c r="J4" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K4" t="str">
-        <v>Catholic</v>
+        <v>Katolik</v>
       </c>
       <c r="L4" t="str">
         <v>Married</v>
@@ -811,7 +811,7 @@
         <v>Active</v>
       </c>
       <c r="X4" t="str">
-        <v>1990-08-05</v>
+        <v>05/08/1990</v>
       </c>
       <c r="Y4" t="str">
         <v>PKWTT</v>
@@ -820,7 +820,7 @@
         <v>-</v>
       </c>
       <c r="AA4" t="str">
-        <v>1990-08-05</v>
+        <v>05/08/1990</v>
       </c>
       <c r="AB4" t="str">
         <v/>
@@ -879,13 +879,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I5" t="str">
-        <v>1959-10-02</v>
+        <v>02/10/1959</v>
       </c>
       <c r="J5" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K5" t="str">
-        <v>Catholic</v>
+        <v>Katolik</v>
       </c>
       <c r="L5" t="str">
         <v>Married</v>
@@ -924,7 +924,7 @@
         <v>Active</v>
       </c>
       <c r="X5" t="str">
-        <v>1990-08-06</v>
+        <v>06/08/1990</v>
       </c>
       <c r="Y5" t="str">
         <v>PKWTT</v>
@@ -933,7 +933,7 @@
         <v>-</v>
       </c>
       <c r="AA5" t="str">
-        <v>1990-08-06</v>
+        <v>06/08/1990</v>
       </c>
       <c r="AB5" t="str">
         <v/>
@@ -992,13 +992,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I6" t="str">
-        <v>1962-09-01</v>
+        <v>01/09/1962</v>
       </c>
       <c r="J6" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K6" t="str">
-        <v>Catholic</v>
+        <v>Katolik</v>
       </c>
       <c r="L6" t="str">
         <v>Single</v>
@@ -1037,7 +1037,7 @@
         <v>Active</v>
       </c>
       <c r="X6" t="str">
-        <v>1990-08-07</v>
+        <v>07/08/1990</v>
       </c>
       <c r="Y6" t="str">
         <v>PKWTT</v>
@@ -1046,7 +1046,7 @@
         <v>-</v>
       </c>
       <c r="AA6" t="str">
-        <v>1990-08-07</v>
+        <v>07/08/1990</v>
       </c>
       <c r="AB6" t="str">
         <v/>
@@ -1105,10 +1105,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I7" t="str">
-        <v>1986-09-29</v>
+        <v>29/09/1986</v>
       </c>
       <c r="J7" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K7" t="str">
         <v>Islam</v>
@@ -1150,7 +1150,7 @@
         <v>Active</v>
       </c>
       <c r="X7" t="str">
-        <v>2020-06-15</v>
+        <v>15/06/2020</v>
       </c>
       <c r="Y7" t="str">
         <v>PKWTT</v>
@@ -1159,7 +1159,7 @@
         <v>-</v>
       </c>
       <c r="AA7" t="str">
-        <v>2020-06-15</v>
+        <v>15/06/2020</v>
       </c>
       <c r="AB7" t="str">
         <v/>
@@ -1218,13 +1218,13 @@
         <v>Singapura</v>
       </c>
       <c r="I8" t="str">
-        <v>1994-03-18</v>
+        <v>18/03/1994</v>
       </c>
       <c r="J8" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K8" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L8" t="str">
         <v>Married</v>
@@ -1263,7 +1263,7 @@
         <v>Active</v>
       </c>
       <c r="X8" t="str">
-        <v>2020-04-20</v>
+        <v>20/04/2020</v>
       </c>
       <c r="Y8" t="str">
         <v>PKWTT</v>
@@ -1272,7 +1272,7 @@
         <v>-</v>
       </c>
       <c r="AA8" t="str">
-        <v>2020-04-20</v>
+        <v>20/04/2020</v>
       </c>
       <c r="AB8" t="str">
         <v/>
@@ -1331,13 +1331,13 @@
         <v>Medan</v>
       </c>
       <c r="I9" t="str">
-        <v>1987-10-06</v>
+        <v>06/10/1987</v>
       </c>
       <c r="J9" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K9" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L9" t="str">
         <v>Single</v>
@@ -1376,7 +1376,7 @@
         <v>Active</v>
       </c>
       <c r="X9" t="str">
-        <v>2019-11-01</v>
+        <v>01/11/2019</v>
       </c>
       <c r="Y9" t="str">
         <v>PKWTT</v>
@@ -1385,7 +1385,7 @@
         <v>-</v>
       </c>
       <c r="AA9" t="str">
-        <v>2019-11-01</v>
+        <v>01/11/2019</v>
       </c>
       <c r="AB9" t="str">
         <v/>
@@ -1444,10 +1444,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I10" t="str">
-        <v>1974-12-16</v>
+        <v>16/12/1974</v>
       </c>
       <c r="J10" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K10" t="str">
         <v>Islam</v>
@@ -1489,7 +1489,7 @@
         <v>Active</v>
       </c>
       <c r="X10" t="str">
-        <v>1996-11-20</v>
+        <v>20/11/1996</v>
       </c>
       <c r="Y10" t="str">
         <v>PKWTT</v>
@@ -1498,7 +1498,7 @@
         <v>-</v>
       </c>
       <c r="AA10" t="str">
-        <v>1996-11-20</v>
+        <v>20/11/1996</v>
       </c>
       <c r="AB10" t="str">
         <v/>
@@ -1557,10 +1557,10 @@
         <v>Kediri</v>
       </c>
       <c r="I11" t="str">
-        <v>1969-12-17</v>
+        <v>17/12/1969</v>
       </c>
       <c r="J11" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K11" t="str">
         <v>Islam</v>
@@ -1602,7 +1602,7 @@
         <v>Active</v>
       </c>
       <c r="X11" t="str">
-        <v>1999-07-19</v>
+        <v>19/07/1999</v>
       </c>
       <c r="Y11" t="str">
         <v>PKWTT</v>
@@ -1611,7 +1611,7 @@
         <v>-</v>
       </c>
       <c r="AA11" t="str">
-        <v>1999-07-19</v>
+        <v>19/07/1999</v>
       </c>
       <c r="AB11" t="str">
         <v/>
@@ -1670,13 +1670,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I12" t="str">
-        <v>1973-12-24</v>
+        <v>24/12/1973</v>
       </c>
       <c r="J12" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K12" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L12" t="str">
         <v>Married</v>
@@ -1715,7 +1715,7 @@
         <v>Active</v>
       </c>
       <c r="X12" t="str">
-        <v>1996-05-01</v>
+        <v>01/05/1996</v>
       </c>
       <c r="Y12" t="str">
         <v>PKWTT</v>
@@ -1724,7 +1724,7 @@
         <v>-</v>
       </c>
       <c r="AA12" t="str">
-        <v>1996-05-01</v>
+        <v>01/05/1996</v>
       </c>
       <c r="AB12" t="str">
         <v/>
@@ -1783,13 +1783,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I13" t="str">
-        <v>1965-10-07</v>
+        <v>07/10/1965</v>
       </c>
       <c r="J13" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K13" t="str">
-        <v>Catholic</v>
+        <v>Katolik</v>
       </c>
       <c r="L13" t="str">
         <v>Married</v>
@@ -1828,7 +1828,7 @@
         <v>Active</v>
       </c>
       <c r="X13" t="str">
-        <v>1999-09-01</v>
+        <v>01/09/1999</v>
       </c>
       <c r="Y13" t="str">
         <v>PKWTT</v>
@@ -1837,7 +1837,7 @@
         <v>-</v>
       </c>
       <c r="AA13" t="str">
-        <v>1999-09-01</v>
+        <v>01/09/1999</v>
       </c>
       <c r="AB13" t="str">
         <v/>
@@ -1896,10 +1896,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I14" t="str">
-        <v>1969-04-18</v>
+        <v>18/04/1969</v>
       </c>
       <c r="J14" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K14" t="str">
         <v>Buddha</v>
@@ -1941,7 +1941,7 @@
         <v>Active</v>
       </c>
       <c r="X14" t="str">
-        <v>1999-08-04</v>
+        <v>04/08/1999</v>
       </c>
       <c r="Y14" t="str">
         <v>PKWTT</v>
@@ -1950,7 +1950,7 @@
         <v>-</v>
       </c>
       <c r="AA14" t="str">
-        <v>1999-08-04</v>
+        <v>04/08/1999</v>
       </c>
       <c r="AB14" t="str">
         <v/>
@@ -2009,13 +2009,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I15" t="str">
-        <v>1986-09-22</v>
+        <v>22/09/1986</v>
       </c>
       <c r="J15" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K15" t="str">
-        <v>Catholic</v>
+        <v>Katolik</v>
       </c>
       <c r="L15" t="str">
         <v>Married</v>
@@ -2054,7 +2054,7 @@
         <v>Active</v>
       </c>
       <c r="X15" t="str">
-        <v>2013-07-29</v>
+        <v>29/07/2013</v>
       </c>
       <c r="Y15" t="str">
         <v>PKWTT</v>
@@ -2063,7 +2063,7 @@
         <v>-</v>
       </c>
       <c r="AA15" t="str">
-        <v>2013-07-29</v>
+        <v>29/07/2013</v>
       </c>
       <c r="AB15" t="str">
         <v/>
@@ -2122,10 +2122,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I16" t="str">
-        <v>1969-05-29</v>
+        <v>29/05/1969</v>
       </c>
       <c r="J16" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K16" t="str">
         <v>Islam</v>
@@ -2167,7 +2167,7 @@
         <v>Active</v>
       </c>
       <c r="X16" t="str">
-        <v>1991-10-01</v>
+        <v>01/10/1991</v>
       </c>
       <c r="Y16" t="str">
         <v>PKWTT</v>
@@ -2176,7 +2176,7 @@
         <v>-</v>
       </c>
       <c r="AA16" t="str">
-        <v>1991-10-01</v>
+        <v>01/10/1991</v>
       </c>
       <c r="AB16" t="str">
         <v/>
@@ -2235,10 +2235,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I17" t="str">
-        <v>1987-07-27</v>
+        <v>27/07/1987</v>
       </c>
       <c r="J17" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K17" t="str">
         <v>Islam</v>
@@ -2280,7 +2280,7 @@
         <v>Active</v>
       </c>
       <c r="X17" t="str">
-        <v>2021-07-01</v>
+        <v>01/07/2021</v>
       </c>
       <c r="Y17" t="str">
         <v>PKWTT</v>
@@ -2289,7 +2289,7 @@
         <v>-</v>
       </c>
       <c r="AA17" t="str">
-        <v>2021-07-01</v>
+        <v>01/07/2021</v>
       </c>
       <c r="AB17" t="str">
         <v/>
@@ -2348,13 +2348,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I18" t="str">
-        <v>1965-01-28</v>
+        <v>28/01/1965</v>
       </c>
       <c r="J18" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K18" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L18" t="str">
         <v>Married</v>
@@ -2393,7 +2393,7 @@
         <v>Active</v>
       </c>
       <c r="X18" t="str">
-        <v>2015-01-29</v>
+        <v>29/01/2015</v>
       </c>
       <c r="Y18" t="str">
         <v>PKWTT</v>
@@ -2402,7 +2402,7 @@
         <v>-</v>
       </c>
       <c r="AA18" t="str">
-        <v>2015-01-29</v>
+        <v>29/01/2015</v>
       </c>
       <c r="AB18" t="str">
         <v/>
@@ -2461,13 +2461,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I19" t="str">
-        <v>1986-08-04</v>
+        <v>04/08/1986</v>
       </c>
       <c r="J19" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K19" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L19" t="str">
         <v>Married</v>
@@ -2506,7 +2506,7 @@
         <v>Active</v>
       </c>
       <c r="X19" t="str">
-        <v>2014-11-24</v>
+        <v>24/11/2014</v>
       </c>
       <c r="Y19" t="str">
         <v>PKWTT</v>
@@ -2515,7 +2515,7 @@
         <v>-</v>
       </c>
       <c r="AA19" t="str">
-        <v>2014-11-24</v>
+        <v>24/11/2014</v>
       </c>
       <c r="AB19" t="str">
         <v/>
@@ -2574,13 +2574,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I20" t="str">
-        <v>1987-03-03</v>
+        <v>03/03/1987</v>
       </c>
       <c r="J20" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K20" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L20" t="str">
         <v>Single</v>
@@ -2619,7 +2619,7 @@
         <v>Active</v>
       </c>
       <c r="X20" t="str">
-        <v>2014-04-01</v>
+        <v>01/04/2014</v>
       </c>
       <c r="Y20" t="str">
         <v>PKWTT</v>
@@ -2628,7 +2628,7 @@
         <v>-</v>
       </c>
       <c r="AA20" t="str">
-        <v>2014-04-01</v>
+        <v>01/04/2014</v>
       </c>
       <c r="AB20" t="str">
         <v/>
@@ -2687,13 +2687,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I21" t="str">
-        <v>1993-05-09</v>
+        <v>09/05/1993</v>
       </c>
       <c r="J21" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K21" t="str">
-        <v>Catholic</v>
+        <v>Katolik</v>
       </c>
       <c r="L21" t="str">
         <v>Married</v>
@@ -2732,7 +2732,7 @@
         <v>Active</v>
       </c>
       <c r="X21" t="str">
-        <v>2021-03-08</v>
+        <v>08/03/2021</v>
       </c>
       <c r="Y21" t="str">
         <v>PKWTT</v>
@@ -2741,7 +2741,7 @@
         <v>-</v>
       </c>
       <c r="AA21" t="str">
-        <v>2021-03-08</v>
+        <v>08/03/2021</v>
       </c>
       <c r="AB21" t="str">
         <v/>
@@ -2800,13 +2800,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I22" t="str">
-        <v>1992-11-24</v>
+        <v>24/11/1992</v>
       </c>
       <c r="J22" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K22" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L22" t="str">
         <v>Single</v>
@@ -2845,7 +2845,7 @@
         <v>Active</v>
       </c>
       <c r="X22" t="str">
-        <v>2016-08-28</v>
+        <v>28/08/2016</v>
       </c>
       <c r="Y22" t="str">
         <v>PKWTT</v>
@@ -2854,7 +2854,7 @@
         <v>-</v>
       </c>
       <c r="AA22" t="str">
-        <v>2016-08-28</v>
+        <v>28/08/2016</v>
       </c>
       <c r="AB22" t="str">
         <v/>
@@ -2913,13 +2913,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I23" t="str">
-        <v>1988-06-25</v>
+        <v>25/06/1988</v>
       </c>
       <c r="J23" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K23" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L23" t="str">
         <v>Married</v>
@@ -2958,7 +2958,7 @@
         <v>Active</v>
       </c>
       <c r="X23" t="str">
-        <v>2018-07-30</v>
+        <v>30/07/2018</v>
       </c>
       <c r="Y23" t="str">
         <v>PKWTT</v>
@@ -2967,7 +2967,7 @@
         <v>-</v>
       </c>
       <c r="AA23" t="str">
-        <v>2018-07-30</v>
+        <v>30/07/2018</v>
       </c>
       <c r="AB23" t="str">
         <v/>
@@ -3026,10 +3026,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I24" t="str">
-        <v>1983-03-19</v>
+        <v>19/03/1983</v>
       </c>
       <c r="J24" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K24" t="str">
         <v>Islam</v>
@@ -3071,7 +3071,7 @@
         <v>Active</v>
       </c>
       <c r="X24" t="str">
-        <v>2006-01-16</v>
+        <v>16/01/2006</v>
       </c>
       <c r="Y24" t="str">
         <v>PKWTT</v>
@@ -3080,7 +3080,7 @@
         <v>-</v>
       </c>
       <c r="AA24" t="str">
-        <v>2006-01-16</v>
+        <v>16/01/2006</v>
       </c>
       <c r="AB24" t="str">
         <v/>
@@ -3139,13 +3139,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I25" t="str">
-        <v>1959-09-13</v>
+        <v>13/09/1959</v>
       </c>
       <c r="J25" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K25" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L25" t="str">
         <v>Married</v>
@@ -3188,7 +3188,7 @@
         <v>Active</v>
       </c>
       <c r="X25" t="str">
-        <v>1997-09-12</v>
+        <v>12/09/1997</v>
       </c>
       <c r="Y25" t="str">
         <v>PKWTT</v>
@@ -3197,7 +3197,7 @@
         <v>-</v>
       </c>
       <c r="AA25" t="str">
-        <v>1997-09-12</v>
+        <v>12/09/1997</v>
       </c>
       <c r="AB25" t="str">
         <v/>
@@ -3256,10 +3256,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I26" t="str">
-        <v>1990-11-09</v>
+        <v>09/11/1990</v>
       </c>
       <c r="J26" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K26" t="str">
         <v>Islam</v>
@@ -3301,7 +3301,7 @@
         <v>Active</v>
       </c>
       <c r="X26" t="str">
-        <v>2016-04-15</v>
+        <v>15/04/2016</v>
       </c>
       <c r="Y26" t="str">
         <v>PKWTT</v>
@@ -3310,7 +3310,7 @@
         <v>-</v>
       </c>
       <c r="AA26" t="str">
-        <v>2016-04-15</v>
+        <v>15/04/2016</v>
       </c>
       <c r="AB26" t="str">
         <v/>
@@ -3369,13 +3369,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I27" t="str">
-        <v>1989-10-12</v>
+        <v>12/10/1989</v>
       </c>
       <c r="J27" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K27" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L27" t="str">
         <v>Married</v>
@@ -3414,7 +3414,7 @@
         <v>Active</v>
       </c>
       <c r="X27" t="str">
-        <v>2020-01-03</v>
+        <v>03/01/2020</v>
       </c>
       <c r="Y27" t="str">
         <v>PKWTT</v>
@@ -3423,7 +3423,7 @@
         <v>-</v>
       </c>
       <c r="AA27" t="str">
-        <v>2020-01-03</v>
+        <v>03/01/2020</v>
       </c>
       <c r="AB27" t="str">
         <v/>
@@ -3482,13 +3482,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I28" t="str">
-        <v>1994-10-11</v>
+        <v>11/10/1994</v>
       </c>
       <c r="J28" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K28" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L28" t="str">
         <v>Married</v>
@@ -3527,7 +3527,7 @@
         <v>Active</v>
       </c>
       <c r="X28" t="str">
-        <v>2019-06-24</v>
+        <v>24/06/2019</v>
       </c>
       <c r="Y28" t="str">
         <v>PKWTT</v>
@@ -3536,7 +3536,7 @@
         <v>-</v>
       </c>
       <c r="AA28" t="str">
-        <v>2019-06-24</v>
+        <v>24/06/2019</v>
       </c>
       <c r="AB28" t="str">
         <v/>
@@ -3595,13 +3595,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I29" t="str">
-        <v>1970-06-08</v>
+        <v>08/06/1970</v>
       </c>
       <c r="J29" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K29" t="str">
-        <v>Catholic</v>
+        <v>Katolik</v>
       </c>
       <c r="L29" t="str">
         <v>Widow</v>
@@ -3640,7 +3640,7 @@
         <v>Active</v>
       </c>
       <c r="X29" t="str">
-        <v>2008-05-01</v>
+        <v>01/05/2008</v>
       </c>
       <c r="Y29" t="str">
         <v>PKWTT</v>
@@ -3649,7 +3649,7 @@
         <v>-</v>
       </c>
       <c r="AA29" t="str">
-        <v>2008-05-01</v>
+        <v>01/05/2008</v>
       </c>
       <c r="AB29" t="str">
         <v/>
@@ -3708,13 +3708,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I30" t="str">
-        <v>1992-01-03</v>
+        <v>03/01/1992</v>
       </c>
       <c r="J30" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K30" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L30" t="str">
         <v>Married</v>
@@ -3753,7 +3753,7 @@
         <v>Active</v>
       </c>
       <c r="X30" t="str">
-        <v>2017-07-13</v>
+        <v>13/07/2017</v>
       </c>
       <c r="Y30" t="str">
         <v>PKWTT</v>
@@ -3762,7 +3762,7 @@
         <v>-</v>
       </c>
       <c r="AA30" t="str">
-        <v>2017-07-13</v>
+        <v>13/07/2017</v>
       </c>
       <c r="AB30" t="str">
         <v/>
@@ -3821,13 +3821,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I31" t="str">
-        <v>1975-12-02</v>
+        <v>02/12/1975</v>
       </c>
       <c r="J31" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K31" t="str">
-        <v>Catholic</v>
+        <v>Katolik</v>
       </c>
       <c r="L31" t="str">
         <v>Married</v>
@@ -3866,7 +3866,7 @@
         <v>Active</v>
       </c>
       <c r="X31" t="str">
-        <v>2011-05-16</v>
+        <v>16/05/2011</v>
       </c>
       <c r="Y31" t="str">
         <v>PKWTT</v>
@@ -3875,7 +3875,7 @@
         <v>-</v>
       </c>
       <c r="AA31" t="str">
-        <v>2011-05-16</v>
+        <v>16/05/2011</v>
       </c>
       <c r="AB31" t="str">
         <v/>
@@ -3934,10 +3934,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I32" t="str">
-        <v>1983-05-07</v>
+        <v>07/05/1983</v>
       </c>
       <c r="J32" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K32" t="str">
         <v>Buddha</v>
@@ -3979,7 +3979,7 @@
         <v>Active</v>
       </c>
       <c r="X32" t="str">
-        <v>2019-01-02</v>
+        <v>02/01/2019</v>
       </c>
       <c r="Y32" t="str">
         <v>PKWTT</v>
@@ -3988,7 +3988,7 @@
         <v>-</v>
       </c>
       <c r="AA32" t="str">
-        <v>2019-01-02</v>
+        <v>02/01/2019</v>
       </c>
       <c r="AB32" t="str">
         <v/>
@@ -4047,13 +4047,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I33" t="str">
-        <v>1989-08-15</v>
+        <v>15/08/1989</v>
       </c>
       <c r="J33" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K33" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L33" t="str">
         <v>Single</v>
@@ -4092,7 +4092,7 @@
         <v>Active</v>
       </c>
       <c r="X33" t="str">
-        <v>2013-12-16</v>
+        <v>16/12/2013</v>
       </c>
       <c r="Y33" t="str">
         <v>PKWTT</v>
@@ -4101,7 +4101,7 @@
         <v>-</v>
       </c>
       <c r="AA33" t="str">
-        <v>2013-12-16</v>
+        <v>16/12/2013</v>
       </c>
       <c r="AB33" t="str">
         <v/>
@@ -4160,10 +4160,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I34" t="str">
-        <v>1991-03-04</v>
+        <v>04/03/1991</v>
       </c>
       <c r="J34" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K34" t="str">
         <v>Islam</v>
@@ -4205,7 +4205,7 @@
         <v>Active</v>
       </c>
       <c r="X34" t="str">
-        <v>2012-02-06</v>
+        <v>06/02/2012</v>
       </c>
       <c r="Y34" t="str">
         <v>PKWTT</v>
@@ -4214,7 +4214,7 @@
         <v>-</v>
       </c>
       <c r="AA34" t="str">
-        <v>2012-02-06</v>
+        <v>06/02/2012</v>
       </c>
       <c r="AB34" t="str">
         <v/>
@@ -4273,10 +4273,10 @@
         <v>Madiun</v>
       </c>
       <c r="I35" t="str">
-        <v>1974-03-26</v>
+        <v>26/03/1974</v>
       </c>
       <c r="J35" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K35" t="str">
         <v>Islam</v>
@@ -4318,7 +4318,7 @@
         <v>Active</v>
       </c>
       <c r="X35" t="str">
-        <v>1993-10-29</v>
+        <v>29/10/1993</v>
       </c>
       <c r="Y35" t="str">
         <v>PKWTT</v>
@@ -4327,7 +4327,7 @@
         <v>-</v>
       </c>
       <c r="AA35" t="str">
-        <v>1993-10-29</v>
+        <v>29/10/1993</v>
       </c>
       <c r="AB35" t="str">
         <v/>
@@ -4386,10 +4386,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I36" t="str">
-        <v>1986-09-03</v>
+        <v>03/09/1986</v>
       </c>
       <c r="J36" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K36" t="str">
         <v>Islam</v>
@@ -4431,7 +4431,7 @@
         <v>Active</v>
       </c>
       <c r="X36" t="str">
-        <v>2006-02-27</v>
+        <v>27/02/2006</v>
       </c>
       <c r="Y36" t="str">
         <v>PKWTT</v>
@@ -4440,7 +4440,7 @@
         <v>-</v>
       </c>
       <c r="AA36" t="str">
-        <v>2006-02-27</v>
+        <v>27/02/2006</v>
       </c>
       <c r="AB36" t="str">
         <v/>
@@ -4499,10 +4499,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I37" t="str">
-        <v>1967-01-17</v>
+        <v>17/01/1967</v>
       </c>
       <c r="J37" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K37" t="str">
         <v>Islam</v>
@@ -4544,7 +4544,7 @@
         <v>Active</v>
       </c>
       <c r="X37" t="str">
-        <v>2006-10-31</v>
+        <v>31/10/2006</v>
       </c>
       <c r="Y37" t="str">
         <v>PKWTT</v>
@@ -4553,7 +4553,7 @@
         <v>-</v>
       </c>
       <c r="AA37" t="str">
-        <v>2006-10-31</v>
+        <v>31/10/2006</v>
       </c>
       <c r="AB37" t="str">
         <v/>
@@ -4612,10 +4612,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I38" t="str">
-        <v>1975-01-15</v>
+        <v>15/01/1975</v>
       </c>
       <c r="J38" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K38" t="str">
         <v>Islam</v>
@@ -4657,7 +4657,7 @@
         <v>Active</v>
       </c>
       <c r="X38" t="str">
-        <v>2009-10-21</v>
+        <v>21/10/2009</v>
       </c>
       <c r="Y38" t="str">
         <v>PKWTT</v>
@@ -4666,7 +4666,7 @@
         <v>-</v>
       </c>
       <c r="AA38" t="str">
-        <v>2009-10-21</v>
+        <v>21/10/2009</v>
       </c>
       <c r="AB38" t="str">
         <v/>
@@ -4725,10 +4725,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I39" t="str">
-        <v>1989-10-07</v>
+        <v>07/10/1989</v>
       </c>
       <c r="J39" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K39" t="str">
         <v>Islam</v>
@@ -4770,7 +4770,7 @@
         <v>Active</v>
       </c>
       <c r="X39" t="str">
-        <v>2022-05-09</v>
+        <v>09/05/2022</v>
       </c>
       <c r="Y39" t="str">
         <v>PKWTT</v>
@@ -4779,7 +4779,7 @@
         <v>-</v>
       </c>
       <c r="AA39" t="str">
-        <v>2022-05-09</v>
+        <v>09/05/2022</v>
       </c>
       <c r="AB39" t="str">
         <v/>
@@ -4838,10 +4838,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I40" t="str">
-        <v>1990-05-14</v>
+        <v>14/05/1990</v>
       </c>
       <c r="J40" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K40" t="str">
         <v>Islam</v>
@@ -4883,7 +4883,7 @@
         <v>Active</v>
       </c>
       <c r="X40" t="str">
-        <v>2022-05-09</v>
+        <v>09/05/2022</v>
       </c>
       <c r="Y40" t="str">
         <v>PKWTT</v>
@@ -4892,7 +4892,7 @@
         <v>-</v>
       </c>
       <c r="AA40" t="str">
-        <v>2022-05-09</v>
+        <v>09/05/2022</v>
       </c>
       <c r="AB40" t="str">
         <v/>
@@ -4951,10 +4951,10 @@
         <v>Purwakarta</v>
       </c>
       <c r="I41" t="str">
-        <v>1999-10-22</v>
+        <v>22/10/1999</v>
       </c>
       <c r="J41" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K41" t="str">
         <v>Islam</v>
@@ -4996,7 +4996,7 @@
         <v>Active</v>
       </c>
       <c r="X41" t="str">
-        <v>2022-09-19</v>
+        <v>19/09/2022</v>
       </c>
       <c r="Y41" t="str">
         <v>PKWTT</v>
@@ -5005,7 +5005,7 @@
         <v>-</v>
       </c>
       <c r="AA41" t="str">
-        <v>2022-09-19</v>
+        <v>19/09/2022</v>
       </c>
       <c r="AB41" t="str">
         <v/>
@@ -5064,13 +5064,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I42" t="str">
-        <v>1978-12-19</v>
+        <v>19/12/1978</v>
       </c>
       <c r="J42" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K42" t="str">
-        <v>Catholic</v>
+        <v>Katolik</v>
       </c>
       <c r="L42" t="str">
         <v>Married</v>
@@ -5109,7 +5109,7 @@
         <v>Active</v>
       </c>
       <c r="X42" t="str">
-        <v>2023-02-06</v>
+        <v>06/02/2023</v>
       </c>
       <c r="Y42" t="str">
         <v>PKWTT</v>
@@ -5118,7 +5118,7 @@
         <v>-</v>
       </c>
       <c r="AA42" t="str">
-        <v>2023-02-06</v>
+        <v>06/02/2023</v>
       </c>
       <c r="AB42" t="str">
         <v/>
@@ -5177,10 +5177,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I43" t="str">
-        <v>1978-06-23</v>
+        <v>23/06/1978</v>
       </c>
       <c r="J43" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K43" t="str">
         <v>Islam</v>
@@ -5222,7 +5222,7 @@
         <v>Active</v>
       </c>
       <c r="X43" t="str">
-        <v>2007-02-12</v>
+        <v>12/02/2007</v>
       </c>
       <c r="Y43" t="str">
         <v>PKWTT</v>
@@ -5231,7 +5231,7 @@
         <v>-</v>
       </c>
       <c r="AA43" t="str">
-        <v>2007-02-12</v>
+        <v>12/02/2007</v>
       </c>
       <c r="AB43" t="str">
         <v/>
@@ -5290,10 +5290,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I44" t="str">
-        <v>1980-02-22</v>
+        <v>22/02/1980</v>
       </c>
       <c r="J44" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K44" t="str">
         <v>Islam</v>
@@ -5335,7 +5335,7 @@
         <v>Active</v>
       </c>
       <c r="X44" t="str">
-        <v>2009-11-13</v>
+        <v>13/11/2009</v>
       </c>
       <c r="Y44" t="str">
         <v>PKWTT</v>
@@ -5344,7 +5344,7 @@
         <v>-</v>
       </c>
       <c r="AA44" t="str">
-        <v>2009-11-13</v>
+        <v>13/11/2009</v>
       </c>
       <c r="AB44" t="str">
         <v/>
@@ -5403,13 +5403,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I45" t="str">
-        <v>1992-09-17</v>
+        <v>17/09/1992</v>
       </c>
       <c r="J45" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K45" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L45" t="str">
         <v>Married</v>
@@ -5448,7 +5448,7 @@
         <v>Active</v>
       </c>
       <c r="X45" t="str">
-        <v>2023-08-01</v>
+        <v>01/08/2023</v>
       </c>
       <c r="Y45" t="str">
         <v>PKWTT</v>
@@ -5457,7 +5457,7 @@
         <v>-</v>
       </c>
       <c r="AA45" t="str">
-        <v>2023-08-01</v>
+        <v>01/08/2023</v>
       </c>
       <c r="AB45" t="str">
         <v/>
@@ -5516,10 +5516,10 @@
         <v>Bogor</v>
       </c>
       <c r="I46" t="str">
-        <v>1995-12-07</v>
+        <v>07/12/1995</v>
       </c>
       <c r="J46" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K46" t="str">
         <v>Islam</v>
@@ -5561,7 +5561,7 @@
         <v>Active</v>
       </c>
       <c r="X46" t="str">
-        <v>2023-08-11</v>
+        <v>11/08/2023</v>
       </c>
       <c r="Y46" t="str">
         <v>PKWTT</v>
@@ -5570,7 +5570,7 @@
         <v>-</v>
       </c>
       <c r="AA46" t="str">
-        <v>2023-08-11</v>
+        <v>11/08/2023</v>
       </c>
       <c r="AB46" t="str">
         <v/>
@@ -5629,10 +5629,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I47" t="str">
-        <v>1999-03-13</v>
+        <v>13/03/1999</v>
       </c>
       <c r="J47" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K47" t="str">
         <v>Buddha</v>
@@ -5674,7 +5674,7 @@
         <v>Active</v>
       </c>
       <c r="X47" t="str">
-        <v>2023-10-20</v>
+        <v>20/10/2023</v>
       </c>
       <c r="Y47" t="str">
         <v>PKWTT</v>
@@ -5683,7 +5683,7 @@
         <v>-</v>
       </c>
       <c r="AA47" t="str">
-        <v>2023-10-20</v>
+        <v>20/10/2023</v>
       </c>
       <c r="AB47" t="str">
         <v/>
@@ -5742,10 +5742,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I48" t="str">
-        <v>2000-10-02</v>
+        <v>02/10/2000</v>
       </c>
       <c r="J48" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K48" t="str">
         <v>Islam</v>
@@ -5787,7 +5787,7 @@
         <v>Active</v>
       </c>
       <c r="X48" t="str">
-        <v>2024-01-09</v>
+        <v>09/01/2024</v>
       </c>
       <c r="Y48" t="str">
         <v>PKWTT</v>
@@ -5796,7 +5796,7 @@
         <v>-</v>
       </c>
       <c r="AA48" t="str">
-        <v>2024-01-09</v>
+        <v>09/01/2024</v>
       </c>
       <c r="AB48" t="str">
         <v/>
@@ -5855,10 +5855,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I49" t="str">
-        <v>1999-12-09</v>
+        <v>09/12/1999</v>
       </c>
       <c r="J49" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K49" t="str">
         <v>Islam</v>
@@ -5900,7 +5900,7 @@
         <v>Active</v>
       </c>
       <c r="X49" t="str">
-        <v>2024-02-19</v>
+        <v>19/02/2024</v>
       </c>
       <c r="Y49" t="str">
         <v>PKWTT</v>
@@ -5909,7 +5909,7 @@
         <v>-</v>
       </c>
       <c r="AA49" t="str">
-        <v>2024-02-19</v>
+        <v>19/02/2024</v>
       </c>
       <c r="AB49" t="str">
         <v/>
@@ -5968,10 +5968,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I50" t="str">
-        <v>1989-03-02</v>
+        <v>02/03/1989</v>
       </c>
       <c r="J50" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K50" t="str">
         <v>Islam</v>
@@ -6013,7 +6013,7 @@
         <v>Active</v>
       </c>
       <c r="X50" t="str">
-        <v>2025-03-12</v>
+        <v>12/03/2025</v>
       </c>
       <c r="Y50" t="str">
         <v>PKWTT</v>
@@ -6022,7 +6022,7 @@
         <v>-</v>
       </c>
       <c r="AA50" t="str">
-        <v>2025-03-12</v>
+        <v>12/03/2025</v>
       </c>
       <c r="AB50" t="str">
         <v/>
@@ -6081,13 +6081,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I51" t="str">
-        <v>1988-10-09</v>
+        <v>09/10/1988</v>
       </c>
       <c r="J51" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K51" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L51" t="str">
         <v>Married</v>
@@ -6126,7 +6126,7 @@
         <v>Active</v>
       </c>
       <c r="X51" t="str">
-        <v>2024-06-03</v>
+        <v>03/06/2024</v>
       </c>
       <c r="Y51" t="str">
         <v>PKWTT</v>
@@ -6135,7 +6135,7 @@
         <v>-</v>
       </c>
       <c r="AA51" t="str">
-        <v>2024-06-03</v>
+        <v>03/06/2024</v>
       </c>
       <c r="AB51" t="str">
         <v/>
@@ -6194,13 +6194,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I52" t="str">
-        <v>1989-07-29</v>
+        <v>29/07/1989</v>
       </c>
       <c r="J52" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K52" t="str">
-        <v>Catholic</v>
+        <v>Katolik</v>
       </c>
       <c r="L52" t="str">
         <v>Married</v>
@@ -6239,7 +6239,7 @@
         <v>Active</v>
       </c>
       <c r="X52" t="str">
-        <v>2024-09-01</v>
+        <v>01/09/2024</v>
       </c>
       <c r="Y52" t="str">
         <v>PKWTT</v>
@@ -6248,7 +6248,7 @@
         <v>-</v>
       </c>
       <c r="AA52" t="str">
-        <v>2024-09-01</v>
+        <v>01/09/2024</v>
       </c>
       <c r="AB52" t="str">
         <v/>
@@ -6307,10 +6307,10 @@
         <v>Bogor</v>
       </c>
       <c r="I53" t="str">
-        <v>2000-12-27</v>
+        <v>27/12/2000</v>
       </c>
       <c r="J53" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K53" t="str">
         <v>Islam</v>
@@ -6352,7 +6352,7 @@
         <v>Active</v>
       </c>
       <c r="X53" t="str">
-        <v>2024-09-23</v>
+        <v>23/09/2024</v>
       </c>
       <c r="Y53" t="str">
         <v>PKWTT</v>
@@ -6361,7 +6361,7 @@
         <v>-</v>
       </c>
       <c r="AA53" t="str">
-        <v>2024-09-23</v>
+        <v>23/09/2024</v>
       </c>
       <c r="AB53" t="str">
         <v/>
@@ -6420,13 +6420,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I54" t="str">
-        <v>1987-12-04</v>
+        <v>04/12/1987</v>
       </c>
       <c r="J54" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K54" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L54" t="str">
         <v>Single</v>
@@ -6465,7 +6465,7 @@
         <v>Active</v>
       </c>
       <c r="X54" t="str">
-        <v>2024-11-14</v>
+        <v>14/11/2024</v>
       </c>
       <c r="Y54" t="str">
         <v>PKWTT</v>
@@ -6474,7 +6474,7 @@
         <v>-</v>
       </c>
       <c r="AA54" t="str">
-        <v>2024-11-14</v>
+        <v>14/11/2024</v>
       </c>
       <c r="AB54" t="str">
         <v/>
@@ -6533,10 +6533,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I55" t="str">
-        <v>1999-12-15</v>
+        <v>15/12/1999</v>
       </c>
       <c r="J55" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K55" t="str">
         <v>Islam</v>
@@ -6578,7 +6578,7 @@
         <v>Active</v>
       </c>
       <c r="X55" t="str">
-        <v>2025-02-17</v>
+        <v>17/02/2025</v>
       </c>
       <c r="Y55" t="str">
         <v>PKWTT</v>
@@ -6587,7 +6587,7 @@
         <v>-</v>
       </c>
       <c r="AA55" t="str">
-        <v>2025-02-17</v>
+        <v>17/02/2025</v>
       </c>
       <c r="AB55" t="str">
         <v/>
@@ -6646,13 +6646,13 @@
         <v>Pondok Pinang</v>
       </c>
       <c r="I56" t="str">
-        <v>1995-08-01</v>
+        <v>01/08/1995</v>
       </c>
       <c r="J56" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K56" t="str">
-        <v>Catholic</v>
+        <v>Katolik</v>
       </c>
       <c r="L56" t="str">
         <v>Single</v>
@@ -6691,7 +6691,7 @@
         <v>Active</v>
       </c>
       <c r="X56" t="str">
-        <v>2025-04-07</v>
+        <v>07/04/2025</v>
       </c>
       <c r="Y56" t="str">
         <v>PKWTT</v>
@@ -6700,7 +6700,7 @@
         <v>-</v>
       </c>
       <c r="AA56" t="str">
-        <v>2025-04-07</v>
+        <v>07/04/2025</v>
       </c>
       <c r="AB56" t="str">
         <v/>
@@ -6759,13 +6759,13 @@
         <v>Lumban Hariara</v>
       </c>
       <c r="I57" t="str">
-        <v>1987-10-05</v>
+        <v>05/10/1987</v>
       </c>
       <c r="J57" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K57" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L57" t="str">
         <v>Married</v>
@@ -6804,7 +6804,7 @@
         <v>Active</v>
       </c>
       <c r="X57" t="str">
-        <v>2025-04-14</v>
+        <v>14/04/2025</v>
       </c>
       <c r="Y57" t="str">
         <v>PKWTT</v>
@@ -6813,7 +6813,7 @@
         <v>-</v>
       </c>
       <c r="AA57" t="str">
-        <v>2025-04-14</v>
+        <v>14/04/2025</v>
       </c>
       <c r="AB57" t="str">
         <v/>
@@ -6872,10 +6872,10 @@
         <v>Bandung</v>
       </c>
       <c r="I58" t="str">
-        <v>1996-12-10</v>
+        <v>10/12/1996</v>
       </c>
       <c r="J58" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K58" t="str">
         <v>Islam</v>
@@ -6917,7 +6917,7 @@
         <v>Active</v>
       </c>
       <c r="X58" t="str">
-        <v>2025-06-02</v>
+        <v>02/06/2025</v>
       </c>
       <c r="Y58" t="str">
         <v>PKWTT</v>
@@ -6926,7 +6926,7 @@
         <v>-</v>
       </c>
       <c r="AA58" t="str">
-        <v>2025-06-02</v>
+        <v>02/06/2025</v>
       </c>
       <c r="AB58" t="str">
         <v/>
@@ -6985,13 +6985,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I59" t="str">
-        <v>1988-09-12</v>
+        <v>12/09/1988</v>
       </c>
       <c r="J59" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K59" t="str">
-        <v>Catholic</v>
+        <v>Katolik</v>
       </c>
       <c r="L59" t="str">
         <v>Married</v>
@@ -7030,7 +7030,7 @@
         <v>Active</v>
       </c>
       <c r="X59" t="str">
-        <v>2025-06-02</v>
+        <v>02/06/2025</v>
       </c>
       <c r="Y59" t="str">
         <v>PKWTT</v>
@@ -7039,7 +7039,7 @@
         <v>-</v>
       </c>
       <c r="AA59" t="str">
-        <v>2025-06-02</v>
+        <v>02/06/2025</v>
       </c>
       <c r="AB59" t="str">
         <v/>
@@ -7098,10 +7098,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I60" t="str">
-        <v>1989-06-05</v>
+        <v>05/06/1989</v>
       </c>
       <c r="J60" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K60" t="str">
         <v>Buddha</v>
@@ -7143,7 +7143,7 @@
         <v>Active</v>
       </c>
       <c r="X60" t="str">
-        <v>2025-08-04</v>
+        <v>04/08/2025</v>
       </c>
       <c r="Y60" t="str">
         <v>PKWTT</v>
@@ -7152,7 +7152,7 @@
         <v>-</v>
       </c>
       <c r="AA60" t="str">
-        <v>2025-08-04</v>
+        <v>04/08/2025</v>
       </c>
       <c r="AB60" t="str">
         <v/>
@@ -7211,10 +7211,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I61" t="str">
-        <v>2000-11-30</v>
+        <v>30/11/2000</v>
       </c>
       <c r="J61" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K61" t="str">
         <v>Buddha</v>
@@ -7256,7 +7256,7 @@
         <v>Active</v>
       </c>
       <c r="X61" t="str">
-        <v>2025-10-13</v>
+        <v>13/10/2025</v>
       </c>
       <c r="Y61" t="str">
         <v>PKWTT</v>
@@ -7265,7 +7265,7 @@
         <v>-</v>
       </c>
       <c r="AA61" t="str">
-        <v>2025-10-13</v>
+        <v>13/10/2025</v>
       </c>
       <c r="AB61" t="str">
         <v/>
@@ -7324,13 +7324,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I62" t="str">
-        <v>1993-06-15</v>
+        <v>15/06/1993</v>
       </c>
       <c r="J62" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K62" t="str">
-        <v>Others</v>
+        <v>Lainnya</v>
       </c>
       <c r="L62" t="str">
         <v>Single</v>
@@ -7369,7 +7369,7 @@
         <v>Active</v>
       </c>
       <c r="X62" t="str">
-        <v>2025-12-15</v>
+        <v>15/12/2025</v>
       </c>
       <c r="Y62" t="str">
         <v>PKWTT</v>
@@ -7378,7 +7378,7 @@
         <v>-</v>
       </c>
       <c r="AA62" t="str">
-        <v>2025-12-15</v>
+        <v>15/12/2025</v>
       </c>
       <c r="AB62" t="str">
         <v/>
@@ -7437,13 +7437,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I63" t="str">
-        <v>1998-03-12</v>
+        <v>12/03/1998</v>
       </c>
       <c r="J63" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K63" t="str">
-        <v>Catholic</v>
+        <v>Katolik</v>
       </c>
       <c r="L63" t="str">
         <v>Single</v>
@@ -7482,7 +7482,7 @@
         <v>Active</v>
       </c>
       <c r="X63" t="str">
-        <v>2026-02-16</v>
+        <v>16/02/2026</v>
       </c>
       <c r="Y63" t="str">
         <v>PKWTT</v>
@@ -7491,7 +7491,7 @@
         <v>-</v>
       </c>
       <c r="AA63" t="str">
-        <v>2026-02-16</v>
+        <v>16/02/2026</v>
       </c>
       <c r="AB63" t="str">
         <v/>
@@ -7550,10 +7550,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I64" t="str">
-        <v>1986-05-21</v>
+        <v>21/05/1986</v>
       </c>
       <c r="J64" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K64" t="str">
         <v>Islam</v>
@@ -7595,7 +7595,7 @@
         <v>Active</v>
       </c>
       <c r="X64" t="str">
-        <v>2026-04-17</v>
+        <v>17/04/2026</v>
       </c>
       <c r="Y64" t="str">
         <v>PKWTT</v>
@@ -7604,7 +7604,7 @@
         <v>-</v>
       </c>
       <c r="AA64" t="str">
-        <v>2026-04-17</v>
+        <v>17/04/2026</v>
       </c>
       <c r="AB64" t="str">
         <v/>
@@ -7663,13 +7663,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I65" t="str">
-        <v>1999-02-24</v>
+        <v>24/02/1999</v>
       </c>
       <c r="J65" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K65" t="str">
-        <v>Catholic</v>
+        <v>Katolik</v>
       </c>
       <c r="L65" t="str">
         <v>Single</v>
@@ -7708,7 +7708,7 @@
         <v>Active</v>
       </c>
       <c r="X65" t="str">
-        <v>2026-05-15</v>
+        <v>15/05/2026</v>
       </c>
       <c r="Y65" t="str">
         <v>PKWTT</v>
@@ -7717,7 +7717,7 @@
         <v>-</v>
       </c>
       <c r="AA65" t="str">
-        <v>2026-05-15</v>
+        <v>15/05/2026</v>
       </c>
       <c r="AB65" t="str">
         <v/>
@@ -7776,10 +7776,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I66" t="str">
-        <v>1979-12-07</v>
+        <v>07/12/1979</v>
       </c>
       <c r="J66" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K66" t="str">
         <v>Islam</v>
@@ -7821,7 +7821,7 @@
         <v>Active</v>
       </c>
       <c r="X66" t="str">
-        <v>2026-05-18</v>
+        <v>18/05/2026</v>
       </c>
       <c r="Y66" t="str">
         <v>PKWT</v>
@@ -7830,10 +7830,10 @@
         <v>-</v>
       </c>
       <c r="AA66" t="str">
-        <v>2026-05-18</v>
+        <v>18/05/2026</v>
       </c>
       <c r="AB66" t="str">
-        <v>2026-11-17</v>
+        <v>17/11/2026</v>
       </c>
       <c r="AC66" t="str">
         <v>Active</v>
@@ -7889,10 +7889,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I67" t="str">
-        <v>2003-04-23</v>
+        <v>23/04/2003</v>
       </c>
       <c r="J67" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K67" t="str">
         <v>Islam</v>
@@ -7934,7 +7934,7 @@
         <v>Active</v>
       </c>
       <c r="X67" t="str">
-        <v>2026-07-06</v>
+        <v>06/07/2026</v>
       </c>
       <c r="Y67" t="str">
         <v>PKWT</v>
@@ -7943,10 +7943,10 @@
         <v>-</v>
       </c>
       <c r="AA67" t="str">
-        <v>2026-07-06</v>
+        <v>06/07/2026</v>
       </c>
       <c r="AB67" t="str">
-        <v>2027-01-05</v>
+        <v>05/01/2027</v>
       </c>
       <c r="AC67" t="str">
         <v>Active</v>
@@ -8002,10 +8002,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I68" t="str">
-        <v>1979-12-06</v>
+        <v>06/12/1979</v>
       </c>
       <c r="J68" t="str">
-        <v>Male</v>
+        <v>Laki-laki</v>
       </c>
       <c r="K68" t="str">
         <v>Islam</v>
@@ -8047,7 +8047,7 @@
         <v>Active</v>
       </c>
       <c r="X68" t="str">
-        <v>2026-07-08</v>
+        <v>08/07/2026</v>
       </c>
       <c r="Y68" t="str">
         <v>PKWT</v>
@@ -8056,10 +8056,10 @@
         <v>-</v>
       </c>
       <c r="AA68" t="str">
-        <v>2026-07-08</v>
+        <v>08/07/2026</v>
       </c>
       <c r="AB68" t="str">
-        <v>2027-07-07</v>
+        <v>07/07/2027</v>
       </c>
       <c r="AC68" t="str">
         <v>Active</v>
@@ -8115,10 +8115,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I69" t="str">
-        <v>2000-04-17</v>
+        <v>17/04/2000</v>
       </c>
       <c r="J69" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K69" t="str">
         <v>Buddha</v>
@@ -8160,7 +8160,7 @@
         <v>Active</v>
       </c>
       <c r="X69" t="str">
-        <v>2026-07-27</v>
+        <v>27/07/2026</v>
       </c>
       <c r="Y69" t="str">
         <v>Probation</v>
@@ -8169,10 +8169,10 @@
         <v>-</v>
       </c>
       <c r="AA69" t="str">
-        <v>2026-07-27</v>
+        <v>27/07/2026</v>
       </c>
       <c r="AB69" t="str">
-        <v>2026-10-26</v>
+        <v>26/10/2026</v>
       </c>
       <c r="AC69" t="str">
         <v>Active</v>
@@ -8228,13 +8228,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I70" t="str">
-        <v>1992-06-09</v>
+        <v>09/06/1992</v>
       </c>
       <c r="J70" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K70" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L70" t="str">
         <v>Single</v>
@@ -8273,7 +8273,7 @@
         <v>Active</v>
       </c>
       <c r="X70" t="str">
-        <v>2026-08-10</v>
+        <v>10/08/2026</v>
       </c>
       <c r="Y70" t="str">
         <v>Probation</v>
@@ -8282,10 +8282,10 @@
         <v>-</v>
       </c>
       <c r="AA70" t="str">
-        <v>2026-08-10</v>
+        <v>10/08/2026</v>
       </c>
       <c r="AB70" t="str">
-        <v>2026-11-09</v>
+        <v>09/11/2026</v>
       </c>
       <c r="AC70" t="str">
         <v>Active</v>
@@ -8341,13 +8341,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I71" t="str">
-        <v>2001-09-06</v>
+        <v>06/09/2001</v>
       </c>
       <c r="J71" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K71" t="str">
-        <v>Catholic</v>
+        <v>Katolik</v>
       </c>
       <c r="L71" t="str">
         <v>Single</v>
@@ -8386,7 +8386,7 @@
         <v>Active</v>
       </c>
       <c r="X71" t="str">
-        <v>2026-08-18</v>
+        <v>18/08/2026</v>
       </c>
       <c r="Y71" t="str">
         <v>Probation</v>
@@ -8395,10 +8395,10 @@
         <v>-</v>
       </c>
       <c r="AA71" t="str">
-        <v>2026-08-18</v>
+        <v>18/08/2026</v>
       </c>
       <c r="AB71" t="str">
-        <v>2026-11-17</v>
+        <v>17/11/2026</v>
       </c>
       <c r="AC71" t="str">
         <v>Active</v>
@@ -8454,13 +8454,13 @@
         <v>Jakarta</v>
       </c>
       <c r="I72" t="str">
-        <v>1995-04-11</v>
+        <v>11/04/1995</v>
       </c>
       <c r="J72" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K72" t="str">
-        <v>Christian</v>
+        <v>Kristen Protestan</v>
       </c>
       <c r="L72" t="str">
         <v>Single</v>
@@ -8499,7 +8499,7 @@
         <v>Active</v>
       </c>
       <c r="X72" t="str">
-        <v>2026-08-20</v>
+        <v>20/08/2026</v>
       </c>
       <c r="Y72" t="str">
         <v>Probation</v>
@@ -8508,10 +8508,10 @@
         <v>-</v>
       </c>
       <c r="AA72" t="str">
-        <v>2026-08-20</v>
+        <v>20/08/2026</v>
       </c>
       <c r="AB72" t="str">
-        <v>2026-11-19</v>
+        <v>19/11/2026</v>
       </c>
       <c r="AC72" t="str">
         <v>Active</v>
@@ -8567,10 +8567,10 @@
         <v>Gianyar</v>
       </c>
       <c r="I73" t="str">
-        <v>2004-07-02</v>
+        <v>02/07/2004</v>
       </c>
       <c r="J73" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K73" t="str">
         <v>Hindu</v>
@@ -8612,7 +8612,7 @@
         <v>Active</v>
       </c>
       <c r="X73" t="str">
-        <v>2026-10-05</v>
+        <v>05/10/2026</v>
       </c>
       <c r="Y73" t="str">
         <v>Probation</v>
@@ -8621,10 +8621,10 @@
         <v>-</v>
       </c>
       <c r="AA73" t="str">
-        <v>2026-10-05</v>
+        <v>05/10/2026</v>
       </c>
       <c r="AB73" t="str">
-        <v>2027-01-04</v>
+        <v>04/01/2027</v>
       </c>
       <c r="AC73" t="str">
         <v>Active</v>
@@ -8680,10 +8680,10 @@
         <v>Jakarta</v>
       </c>
       <c r="I74" t="str">
-        <v>1999-10-28</v>
+        <v>28/10/1999</v>
       </c>
       <c r="J74" t="str">
-        <v>Female</v>
+        <v>Perempuan</v>
       </c>
       <c r="K74" t="str">
         <v>Islam</v>
@@ -8725,7 +8725,7 @@
         <v>Active</v>
       </c>
       <c r="X74" t="str">
-        <v>2026-09-21</v>
+        <v>21/09/2026</v>
       </c>
       <c r="Y74" t="str">
         <v>PKWT</v>
@@ -8734,10 +8734,10 @@
         <v>-</v>
       </c>
       <c r="AA74" t="str">
-        <v>2026-09-21</v>
+        <v>21/09/2026</v>
       </c>
       <c r="AB74" t="str">
-        <v>2027-03-20</v>
+        <v>20/03/2027</v>
       </c>
       <c r="AC74" t="str">
         <v>Active</v>

</xml_diff>